<commit_message>
Update pinned FASTA references and bilingual catalogue to v1.2.0
</commit_message>
<xml_diff>
--- a/catalogue/benchmark_dataset.xlsx
+++ b/catalogue/benchmark_dataset.xlsx
@@ -26,7 +26,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'fa'!$A$1:$H$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'fa'!$A$1:$M$19</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'fa'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'fq'!$A$2:$Z$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'fq'!$1:$2</definedName>
@@ -601,7 +601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.7109375" customWidth="1" min="1" max="1"/>
@@ -612,6 +612,11 @@
     <col width="35.7109375" customWidth="1" min="6" max="6"/>
     <col width="72.7109375" customWidth="1" min="7" max="7"/>
     <col width="65.7109375" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="65" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="52" customHeight="1">
@@ -637,7 +642,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Reference source link</t>
+          <t>NCBI record</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -652,7 +657,32 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Proposed FASTA download</t>
+          <t>FASTA download</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Expected bytes</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Publisher MD5</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Assembly release date</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Metadata checked date</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Publisher checksum URL</t>
         </is>
       </c>
     </row>
@@ -662,7 +692,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>GRCh38</t>
+          <t>GRCh38.p14</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -672,37 +702,60 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>GCF_000001405.39</t>
+          <t>GCF_000001405.40</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://www.ncbi.nlm.nih.gov/datasets/genome/GCF_000001405.40/</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Direct gzip FASTA route</t>
+          <t>NCBI assembly record; direct gzip FASTA link supplied separately</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Same-species proposal only; sample/strain/target/contig match and FASTA contents unverified.</t>
+          <t>Human reference genome; matching to individual donors has not been checked.</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="78" customHeight="1">
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/000/001/405/GCF_000001405.40_GRCh38.p14/GCF_000001405.40_GRCh38.p14_genomic.fna.gz</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="n">
+        <v>972898531</v>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>c30471567037b2b2389d43c908c653e1</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>2022-02-03</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/000/001/405/GCF_000001405.40_GRCh38.p14/md5checksums.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="95" customHeight="1">
       <c r="A3" s="6" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Sscrofa11.1</t>
+          <t>Sscrofa_HxYL_maternal_Yorkshire_Landrace_v2.0</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -712,27 +765,50 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>GCA_000003025.6</t>
+          <t>GCF_054392235.1</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://www.ncbi.nlm.nih.gov/datasets/genome/GCF_054392235.1/</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Accession landing page; exact FASTA retrieval remains to be fixed</t>
+          <t>NCBI assembly record; direct gzip FASTA link supplied separately</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Same-species proposal only; sample/strain/target/contig match and FASTA contents unverified.</t>
+          <t>Yorkshire/Landrace pig reference; the selected FASTQ sample's breed has not been established.</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/054/392/235/GCF_054392235.1_Sscrofa_HxYL_maternal_Yorkshire_Landrace_v2.0/GCF_054392235.1_Sscrofa_HxYL_maternal_Yorkshire_Landrace_v2.0_genomic.fna.gz</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="n">
+        <v>796779932</v>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>56b9f3d9c185e35e2410611e424ec6eb</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/054/392/235/GCF_054392235.1_Sscrofa_HxYL_maternal_Yorkshire_Landrace_v2.0/md5checksums.txt</t>
         </is>
       </c>
     </row>
@@ -742,7 +818,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>GRCm38</t>
+          <t>GRCm39</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -752,27 +828,50 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>GCF_000001635.24</t>
+          <t>GCF_000001635.27</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://www.ncbi.nlm.nih.gov/datasets/genome/GCF_000001635.27/</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Direct gzip FASTA route</t>
+          <t>NCBI assembly record; direct gzip FASTA link supplied separately</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Same-species genomic reference proposal for mouse inputs; sample/strain/target match and FASTA contents unverified. For Smart-seq2, transcript/patch equivalence and auxiliary ERCC version are separately unverified.</t>
+          <t>C57BL/6J mouse reference; donor substrain and transcript targets need checking. ERCC spike-ins require a separate reference.</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/000/001/635/GCF_000001635.27_GRCm39/GCF_000001635.27_GRCm39_genomic.fna.gz</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="n">
+        <v>834262758</v>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>c0b0c4c3f54d2b480efe68a18bf7e42b</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>2020-06-24</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/000/001/635/GCF_000001635.27_GRCm39/md5checksums.txt</t>
         </is>
       </c>
     </row>
@@ -782,12 +881,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>ASM584</t>
+          <t>ASM584v2</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Escherichia coli</t>
+          <t>Escherichia coli str. K-12 substr. MG1655</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -797,22 +896,45 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://www.ncbi.nlm.nih.gov/datasets/genome/GCF_000005845.2/</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Direct gzip FASTA route</t>
+          <t>NCBI assembly record; direct gzip FASTA link supplied separately</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Same-species proposal only; sample/strain/target/contig match and FASTA contents unverified.</t>
+          <t>MG1655 reference for the MG1655 input; exact read-to-reference matching has not been measured.</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/000/005/845/GCF_000005845.2_ASM584v2/GCF_000005845.2_ASM584v2_genomic.fna.gz</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>1379902</v>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>c13d459b5caa702ff7e1f26fe44b8ad7</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>2013-09-26</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/000/005/845/GCF_000005845.2_ASM584v2/md5checksums.txt</t>
         </is>
       </c>
     </row>
@@ -822,12 +944,12 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>ASM19595v2 (H37Rv)</t>
+          <t>ASM19595v2</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Mycobacterium tuberculosis</t>
+          <t>Mycobacterium tuberculosis H37Rv</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -837,22 +959,45 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://www.ncbi.nlm.nih.gov/datasets/genome/GCF_000195955.2/</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Direct gzip FASTA route</t>
+          <t>NCBI assembly record; direct gzip FASTA link supplied separately</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Same-species proposal only; sample/strain/target/contig match and FASTA contents unverified.</t>
+          <t>H37Rv reference; the selected sample's exact strain match has not been checked.</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/000/195/955/GCF_000195955.2_ASM19595v2/GCF_000195955.2_ASM19595v2_genomic.fna.gz</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>1277508</v>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>f93726a0a6e57af2bf1173998fbeb546</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>2013-02-01</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/000/195/955/GCF_000195955.2_ASM19595v2/md5checksums.txt</t>
         </is>
       </c>
     </row>
@@ -872,27 +1017,50 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>GCA_000226075.1</t>
+          <t>GCF_000226075.1</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://www.ncbi.nlm.nih.gov/datasets/genome/GCF_000226075.1/</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Direct gzip FASTA route</t>
+          <t>NCBI assembly record; direct gzip FASTA link supplied separately</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Same-species proposal only; sample/strain/target/contig match and FASTA contents unverified.</t>
+          <t>DM 1-3 516 R44 reference for the Altus potato input; these are different cultivars.</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/000/226/075/GCF_000226075.1_SolTub_3.0/GCF_000226075.1_SolTub_3.0_genomic.fna.gz</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>210303167</v>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>6ba91aa204b3a87501ff3ed5564183fd</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>2011-09-19</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/000/226/075/GCF_000226075.1_SolTub_3.0/md5checksums.txt</t>
         </is>
       </c>
     </row>
@@ -907,7 +1075,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Saccharomyces cerevisiae</t>
+          <t>Saccharomyces cerevisiae S288C</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -917,22 +1085,45 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://www.ncbi.nlm.nih.gov/datasets/genome/GCF_000146045.2/</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Direct gzip FASTA route</t>
+          <t>NCBI assembly record; direct gzip FASTA link supplied separately</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Same-species proposal only; sample/strain/target/contig match and FASTA contents unverified.</t>
+          <t>S288C yeast reference; exact strain matching has not been checked.</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/000/146/045/GCF_000146045.2_R64/GCF_000146045.2_R64_genomic.fna.gz</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>3843460</v>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>88c38b957b721dfc50e6c4df03b6242e</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>2014-12-17</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/000/146/045/GCF_000146045.2_R64/md5checksums.txt</t>
         </is>
       </c>
     </row>
@@ -942,37 +1133,60 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>ASM1463603v1</t>
+          <t>AGIS1.0</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Oryza sativa</t>
+          <t>Oryza sativa Japonica Group</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>GCA_014636035.1</t>
+          <t>GCF_034140825.1</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://www.ncbi.nlm.nih.gov/datasets/genome/GCF_034140825.1/</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Direct gzip FASTA route</t>
+          <t>NCBI assembly record; direct gzip FASTA link supplied separately</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Same-species proposal only; sample/strain/target/contig match and FASTA contents unverified.</t>
+          <t>Nipponbare japonica rice reference; cultivars of the two selected rice inputs have not been confirmed.</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/034/140/825/GCF_034140825.1_ASM3414082v1/GCF_034140825.1_ASM3414082v1_genomic.fna.gz</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>120268131</v>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>193a5b81b26b57547b1e4c7be4065b89</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>2023-12-06</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/034/140/825/GCF_034140825.1_ASM3414082v1/md5checksums.txt</t>
         </is>
       </c>
     </row>
@@ -997,22 +1211,45 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://www.ncbi.nlm.nih.gov/datasets/genome/GCF_000001735.4/</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Direct gzip FASTA route</t>
+          <t>NCBI assembly record; direct gzip FASTA link supplied separately</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Same-species proposal only; sample/strain/target/contig match and FASTA contents unverified.</t>
+          <t>Columbia Arabidopsis reference; sample and target matching has not been checked.</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/000/001/735/GCF_000001735.4_TAIR10.1/GCF_000001735.4_TAIR10.1_genomic.fna.gz</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>37482399</v>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>0fed2d7901bf1488f20e7ef6842cd84c</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>2018-03-15</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/000/001/735/GCF_000001735.4_TAIR10.1/md5checksums.txt</t>
         </is>
       </c>
     </row>
@@ -1032,27 +1269,50 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>GCA_902167145.1</t>
+          <t>GCF_902167145.1</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://www.ncbi.nlm.nih.gov/datasets/genome/GCF_902167145.1/</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Direct gzip FASTA route</t>
+          <t>NCBI assembly record; direct gzip FASTA link supplied separately</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Same-species, different-inbred B73 reference for SW1611. Exact sample/cultivar/contig matching and FASTA contents remain unverified.</t>
+          <t>B73 maize reference for SW1611 reads; these are different inbred lines.</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/902/167/145/GCF_902167145.1_Zm-B73-REFERENCE-NAM-5.0/GCF_902167145.1_Zm-B73-REFERENCE-NAM-5.0_genomic.fna.gz</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>650091408</v>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>3fe51a7a675eb0ac410814a41d50c775</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>2020-03-21</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/902/167/145/GCF_902167145.1_Zm-B73-REFERENCE-NAM-5.0/md5checksums.txt</t>
         </is>
       </c>
     </row>
@@ -1077,22 +1337,45 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://www.ncbi.nlm.nih.gov/datasets/genome/GCF_042767895.1/</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Direct gzip FASTA route</t>
+          <t>NCBI assembly record; direct gzip FASTA link supplied separately</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Same-species proposal only; sample/strain/target/contig match and FASTA contents unverified.</t>
+          <t>JL-2024 whiteleg shrimp reference; exact sample matching has not been checked.</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/042/767/895/GCF_042767895.1_ASM4276789v1/GCF_042767895.1_ASM4276789v1_genomic.fna.gz</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>437570644</v>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>2a71288f90309178c725a8ba0657451d</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>2024-10-10</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/042/767/895/GCF_042767895.1_ASM4276789v1/md5checksums.txt</t>
         </is>
       </c>
     </row>
@@ -1112,27 +1395,50 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>GCA_016699485.1</t>
+          <t>GCF_016699485.2</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://www.ncbi.nlm.nih.gov/datasets/genome/GCF_016699485.2/</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Direct gzip FASTA route</t>
+          <t>NCBI assembly record; direct gzip FASTA link supplied separately</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Same-species proposal only; sample/strain/target/contig match and FASTA contents unverified.</t>
+          <t>Broiler maternal chicken reference; matching to the selected laying-hen sample has not been checked.</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/016/699/485/GCF_016699485.2_bGalGal1.mat.broiler.GRCg7b/GCF_016699485.2_bGalGal1.mat.broiler.GRCg7b_genomic.fna.gz</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>327035795</v>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>51291297e6b693d8d73207509cbba6aa</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>2021-01-19</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/016/699/485/GCF_016699485.2_bGalGal1.mat.broiler.GRCg7b/md5checksums.txt</t>
         </is>
       </c>
     </row>
@@ -1157,26 +1463,49 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://www.ncbi.nlm.nih.gov/datasets/genome/GCF_000001215.4/</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Direct gzip FASTA route</t>
+          <t>NCBI assembly record; direct gzip FASTA link supplied separately</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Same-species proposal only; sample/strain/target/contig match and FASTA contents unverified.</t>
+          <t>Drosophila reference; exact sample matching has not been checked.</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="62" customHeight="1">
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/000/001/215/GCF_000001215.4_Release_6_plus_ISO1_MT/GCF_000001215.4_Release_6_plus_ISO1_MT_genomic.fna.gz</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>44235956</v>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>869cf40e4f5c7ca27d04ca9ae7baee4f</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>2014-08-01</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/000/001/215/GCF_000001215.4_Release_6_plus_ISO1_MT/md5checksums.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="95" customHeight="1">
       <c r="A15" s="6" t="n">
         <v>14</v>
       </c>
@@ -1197,24 +1526,37 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://www.ncbi.nlm.nih.gov/nuccore/NC_045512.2</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Accession landing page; exact FASTA retrieval remains to be fixed</t>
+          <t>NCBI nucleotide record; versioned FASTA retrieval link supplied separately</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Same-organism label proposal; isolate/variant/target compatibility untested.</t>
+          <t>Fixed Wuhan-Hu-1 reference; matching to the selected sample and targets has not been checked.</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
-        </is>
-      </c>
+          <t>https://eutils.ncbi.nlm.nih.gov/entrez/eutils/efetch.fcgi?db=nuccore&amp;id=NC_045512.2&amp;rettype=fasta&amp;retmode=text</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="n"/>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>Not recorded</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr"/>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr"/>
     </row>
     <row r="16" ht="126" customHeight="1">
       <c r="A16" s="6" t="n">
@@ -1237,22 +1579,45 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://www.ncbi.nlm.nih.gov/datasets/genome/GCA_900067695.1/</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Direct gzip FASTA route</t>
+          <t>NCBI assembly record; direct gzip FASTA link supplied separately</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Proposed same-species assembly; sample/strain/cultivar/target matching and FASTA content unverified.</t>
+          <t>Norway spruce reference for the targeted input; exact sample and target matching has not been checked.</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCA/900/067/695/GCA_900067695.1_Pabies01/GCA_900067695.1_Pabies01_genomic.fna.gz</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="n">
+        <v>4038780371</v>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>f23f2f85b0302fbbaed95d159e0b6a6f</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>2016-11-09</t>
+        </is>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCA/900/067/695/GCA_900067695.1_Pabies01/md5checksums.txt</t>
         </is>
       </c>
     </row>
@@ -1277,22 +1642,45 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://www.ncbi.nlm.nih.gov/datasets/genome/GCF_001683475.1/</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Direct gzip FASTA route</t>
+          <t>NCBI assembly record; direct gzip FASTA link supplied separately</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Proposed same-species assembly; sample/strain/cultivar/target matching and FASTA content unverified.</t>
+          <t>QQ74 quinoa reference; exact cultivar matching has not been checked.</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/001/683/475/GCF_001683475.1_ASM168347v1/GCF_001683475.1_ASM168347v1_genomic.fna.gz</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="n">
+        <v>395946550</v>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>7ba8333bed6ee71c631410104d735017</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>2017-05-19</t>
+        </is>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/001/683/475/GCF_001683475.1_ASM168347v1/md5checksums.txt</t>
         </is>
       </c>
     </row>
@@ -1317,104 +1705,167 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://www.ncbi.nlm.nih.gov/datasets/genome/GCF_003668045.3/</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Direct gzip FASTA route</t>
+          <t>NCBI assembly record; direct gzip FASTA link supplied separately</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Proposed same-species assembly; sample/strain/cultivar/target matching and FASTA content unverified.</t>
+          <t>17A/GY Chinese hamster reference for the CHO input; cell-line differences have not been measured.</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="78" customHeight="1">
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/003/668/045/GCF_003668045.3_CriGri-PICRH-1.0/GCF_003668045.3_CriGri-PICRH-1.0_genomic.fna.gz</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="n">
+        <v>749193397</v>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>9c7ed3f95a6fe684157ff4480a3ece2d</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>2020-06-11</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/003/668/045/GCF_003668045.3_CriGri-PICRH-1.0/md5checksums.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="95" customHeight="1">
       <c r="A19" s="6" t="n">
         <v>18</v>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Triticum_aestivum_Renan_v2.1</t>
+          <t>IWGSC CS RefSeq v2.1</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Triticum aestivum cultivar Renan</t>
+          <t>Triticum aestivum</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>GCA_937894285.1</t>
+          <t>GCF_018294505.1</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://www.ncbi.nlm.nih.gov/datasets/genome/GCF_018294505.1/</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Accession landing page; exactFASTA object must be chosen later</t>
+          <t>NCBI assembly record; direct gzip FASTA link supplied separately</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Same species, different cultivar: proposed Renan assembly for Thatcher wheat reads; exact matching is unverified.</t>
+          <t>Chinese Spring wheat reference for Thatcher reads; these are different cultivars.</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Open source</t>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/018/294/505/GCF_018294505.1_IWGSC_CS_RefSeq_v2.1/GCF_018294505.1_IWGSC_CS_RefSeq_v2.1_genomic.fna.gz</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="n">
+        <v>4338081367</v>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>13acbd8dfa42164e3143543918e8e6a3</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>2021-05-06</t>
+        </is>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>https://ftp.ncbi.nlm.nih.gov/genomes/all/GCF/018/294/505/GCF_018294505.1_IWGSC_CS_RefSeq_v2.1/md5checksums.txt</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H19"/>
+  <autoFilter ref="A1:M19"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId53"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0"/>
@@ -17946,7 +18397,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>1.1.0; see VERSIONING.md. Verification is dated separately.</t>
+          <t>1.2.0; see VERSIONING.md. Verification is dated separately.</t>
         </is>
       </c>
     </row>
@@ -18030,7 +18481,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>The used reference identities have stable fa IDs and exact versions. Landing pages are not direct FASTA links. Mixture and feature definitions remain unspecified where none was accepted.</t>
+          <t>The 18 reference choices were checked against NCBI on 27 October 2026. Use the current NCBI-designated reference genome for each species, retaining the MG1655 strain for the matching E. coli input. The fixed SARS-CoV-2 reference remains NC_045512.2. A current reference can have an old release date; it is not necessarily the most recently submitted assembly. Exact versions, download links and available publisher MD5 values are listed in the fa sheet and reference table. FASTA files were not downloaded in this update. A species reference does not guarantee a match to the sample, cultivar or transcript targets. Mixed communities and tag libraries have no single genome assigned.</t>
         </is>
       </c>
     </row>
@@ -18423,7 +18874,7 @@
       </c>
       <c r="X3" s="3" t="inlineStr">
         <is>
-          <t>fa ID 1 / GCF_000001405.39</t>
+          <t>fa ID 1 / GCF_000001405.40</t>
         </is>
       </c>
       <c r="Y3" s="3" t="n"/>
@@ -18543,7 +18994,7 @@
       </c>
       <c r="X4" s="3" t="inlineStr">
         <is>
-          <t>fa ID 1 / GCF_000001405.39</t>
+          <t>fa ID 1 / GCF_000001405.40</t>
         </is>
       </c>
       <c r="Y4" s="3" t="n"/>
@@ -18663,7 +19114,7 @@
       </c>
       <c r="X5" s="3" t="inlineStr">
         <is>
-          <t>fa ID 1 / GCF_000001405.39</t>
+          <t>fa ID 1 / GCF_000001405.40</t>
         </is>
       </c>
       <c r="Y5" s="3" t="inlineStr">
@@ -18787,7 +19238,7 @@
       </c>
       <c r="X6" s="3" t="inlineStr">
         <is>
-          <t>fa ID 1 / GCF_000001405.39</t>
+          <t>fa ID 1 / GCF_000001405.40</t>
         </is>
       </c>
       <c r="Y6" s="3" t="inlineStr">
@@ -18911,7 +19362,7 @@
       </c>
       <c r="X7" s="3" t="inlineStr">
         <is>
-          <t>fa ID 1 / GCF_000001405.39</t>
+          <t>fa ID 1 / GCF_000001405.40</t>
         </is>
       </c>
       <c r="Y7" s="3" t="n"/>
@@ -19023,7 +19474,7 @@
       </c>
       <c r="X8" s="3" t="inlineStr">
         <is>
-          <t>fa ID 1 / GCF_000001405.39</t>
+          <t>fa ID 1 / GCF_000001405.40</t>
         </is>
       </c>
       <c r="Y8" s="3" t="inlineStr">
@@ -19147,7 +19598,7 @@
       </c>
       <c r="X9" s="3" t="inlineStr">
         <is>
-          <t>fa ID 1 / GCF_000001405.39</t>
+          <t>fa ID 1 / GCF_000001405.40</t>
         </is>
       </c>
       <c r="Y9" s="3" t="n"/>
@@ -19271,7 +19722,7 @@
       </c>
       <c r="X10" s="3" t="inlineStr">
         <is>
-          <t>fa ID 1 / GCF_000001405.39</t>
+          <t>fa ID 1 / GCF_000001405.40</t>
         </is>
       </c>
       <c r="Y10" s="3" t="inlineStr">
@@ -19395,7 +19846,7 @@
       </c>
       <c r="X11" s="3" t="inlineStr">
         <is>
-          <t>fa ID 1 / GCF_000001405.39</t>
+          <t>fa ID 1 / GCF_000001405.40</t>
         </is>
       </c>
       <c r="Y11" s="3" t="inlineStr">
@@ -19519,7 +19970,7 @@
       </c>
       <c r="X12" s="3" t="inlineStr">
         <is>
-          <t>fa ID 10 / GCA_902167145.1</t>
+          <t>fa ID 10 / GCF_902167145.1</t>
         </is>
       </c>
       <c r="Y12" s="3" t="inlineStr">
@@ -19635,7 +20086,7 @@
       </c>
       <c r="X13" s="3" t="inlineStr">
         <is>
-          <t>fa ID 1 / GCF_000001405.39</t>
+          <t>fa ID 1 / GCF_000001405.40</t>
         </is>
       </c>
       <c r="Y13" s="3" t="inlineStr">
@@ -19991,7 +20442,7 @@
       </c>
       <c r="X16" s="3" t="inlineStr">
         <is>
-          <t>fa ID 2 / GCA_000003025.6</t>
+          <t>fa ID 2 / GCF_054392235.1</t>
         </is>
       </c>
       <c r="Y16" s="3" t="n"/>
@@ -20111,7 +20562,7 @@
       </c>
       <c r="X17" s="3" t="inlineStr">
         <is>
-          <t>fa ID 3 / GCF_000001635.24</t>
+          <t>fa ID 3 / GCF_000001635.27</t>
         </is>
       </c>
       <c r="Y17" s="3" t="inlineStr">
@@ -20235,7 +20686,7 @@
       </c>
       <c r="X18" s="3" t="inlineStr">
         <is>
-          <t>fa ID 18 / GCA_937894285.1</t>
+          <t>fa ID 18 / GCF_018294505.1</t>
         </is>
       </c>
       <c r="Y18" s="3" t="inlineStr">
@@ -20359,7 +20810,7 @@
       </c>
       <c r="X19" s="3" t="inlineStr">
         <is>
-          <t>fa ID 6 / GCA_000226075.1</t>
+          <t>fa ID 6 / GCF_000226075.1</t>
         </is>
       </c>
       <c r="Y19" s="3" t="inlineStr">
@@ -20603,7 +21054,7 @@
       </c>
       <c r="X21" s="3" t="inlineStr">
         <is>
-          <t>fa ID 12 / GCA_016699485.1</t>
+          <t>fa ID 12 / GCF_016699485.2</t>
         </is>
       </c>
       <c r="Y21" s="3" t="n"/>
@@ -20723,7 +21174,7 @@
       </c>
       <c r="X22" s="3" t="inlineStr">
         <is>
-          <t>fa ID 1 / GCF_000001405.39</t>
+          <t>fa ID 1 / GCF_000001405.40</t>
         </is>
       </c>
       <c r="Y22" s="3" t="n"/>
@@ -21091,7 +21542,7 @@
       </c>
       <c r="X25" s="3" t="inlineStr">
         <is>
-          <t>fa ID 1 / GCF_000001405.39</t>
+          <t>fa ID 1 / GCF_000001405.40</t>
         </is>
       </c>
       <c r="Y25" s="3" t="n"/>
@@ -21335,7 +21786,7 @@
       </c>
       <c r="X27" s="3" t="inlineStr">
         <is>
-          <t>fa ID 1 / GCF_000001405.39</t>
+          <t>fa ID 1 / GCF_000001405.40</t>
         </is>
       </c>
       <c r="Y27" s="3" t="n"/>
@@ -21447,7 +21898,7 @@
       </c>
       <c r="X28" s="3" t="inlineStr">
         <is>
-          <t>fa ID 1 / GCF_000001405.39</t>
+          <t>fa ID 1 / GCF_000001405.40</t>
         </is>
       </c>
       <c r="Y28" s="3" t="inlineStr">
@@ -21563,7 +22014,7 @@
       </c>
       <c r="X29" s="3" t="inlineStr">
         <is>
-          <t>fa ID 1 / GCF_000001405.39</t>
+          <t>fa ID 1 / GCF_000001405.40</t>
         </is>
       </c>
       <c r="Y29" s="3" t="inlineStr">
@@ -21679,7 +22130,7 @@
       </c>
       <c r="X30" s="3" t="inlineStr">
         <is>
-          <t>fa ID 1 / GCF_000001405.39</t>
+          <t>fa ID 1 / GCF_000001405.40</t>
         </is>
       </c>
       <c r="Y30" s="3" t="inlineStr">
@@ -21803,7 +22254,7 @@
       </c>
       <c r="X31" s="3" t="inlineStr">
         <is>
-          <t>fa ID 3 / GCF_000001635.24</t>
+          <t>fa ID 3 / GCF_000001635.27</t>
         </is>
       </c>
       <c r="Y31" s="3" t="inlineStr">
@@ -22043,7 +22494,7 @@
       </c>
       <c r="X33" s="3" t="inlineStr">
         <is>
-          <t>fa ID 1 / GCF_000001405.39</t>
+          <t>fa ID 1 / GCF_000001405.40</t>
         </is>
       </c>
       <c r="Y33" s="3" t="inlineStr">
@@ -22279,7 +22730,7 @@
       </c>
       <c r="X35" s="3" t="inlineStr">
         <is>
-          <t>fa ID 1 / GCF_000001405.39</t>
+          <t>fa ID 1 / GCF_000001405.40</t>
         </is>
       </c>
       <c r="Y35" s="3" t="inlineStr">
@@ -22403,7 +22854,7 @@
       </c>
       <c r="X36" s="3" t="inlineStr">
         <is>
-          <t>fa ID 1 / GCF_000001405.39</t>
+          <t>fa ID 1 / GCF_000001405.40</t>
         </is>
       </c>
       <c r="Y36" s="3" t="inlineStr">
@@ -22529,7 +22980,7 @@
       </c>
       <c r="X37" s="3" t="inlineStr">
         <is>
-          <t>fa ID 8 / GCA_014636035.1</t>
+          <t>fa ID 8 / GCF_034140825.1</t>
         </is>
       </c>
       <c r="Y37" s="3" t="n"/>
@@ -22651,7 +23102,7 @@
       </c>
       <c r="X38" s="3" t="inlineStr">
         <is>
-          <t>fa ID 1 / GCF_000001405.39; fa ID 13 / GCF_000001215.4</t>
+          <t>fa ID 1 / GCF_000001405.40; fa ID 13 / GCF_000001215.4</t>
         </is>
       </c>
       <c r="Y38" s="3" t="n"/>
@@ -22879,7 +23330,7 @@
       </c>
       <c r="X40" s="3" t="inlineStr">
         <is>
-          <t>fa ID 1 / GCF_000001405.39</t>
+          <t>fa ID 1 / GCF_000001405.40</t>
         </is>
       </c>
       <c r="Y40" s="3" t="inlineStr">
@@ -22995,7 +23446,7 @@
       </c>
       <c r="X41" s="3" t="inlineStr">
         <is>
-          <t>fa ID 8 / GCA_014636035.1</t>
+          <t>fa ID 8 / GCF_034140825.1</t>
         </is>
       </c>
       <c r="Y41" s="3" t="inlineStr">
@@ -31705,7 +32156,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>This ordinary wheat resequencing run adds a large, polyploid crop genome. Both FASTQ ends of one Thatcher sample are included. The primary study reports about 542.5 billion bases and 35× coverage for this sample; this is a real study input, not a subset made to reach a benchmark size. The proposed Renan assembly is from the same species but a different cultivar.</t>
+          <t>This ordinary wheat resequencing run adds a large, polyploid crop genome. Both FASTQ ends of one Thatcher sample are included. The primary study reports about 542.5 billion bases and 35× coverage for this sample; this is a real study input, not a subset made to reach a benchmark size. The proposed Chinese Spring assembly is from the same species but a different cultivar.</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -31715,7 +32166,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>The proposed reference is Renan, not Thatcher; exact read/reference matching remains unverified. Nominal paired 150-base sequencing is documented, but actual FASTQ lengths, qualities, headers and integrity have not been examined.</t>
+          <t>The proposed reference is Chinese Spring, not Thatcher; exact read/reference matching remains unverified. Nominal paired 150-base sequencing is documented, but actual FASTQ lengths, qualities, headers and integrity have not been examined.</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -32175,7 +32626,7 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>Acquire both listed archive ends and verify integrity and pairing. Keep the exact chosen FASTQ representation and order. Same-species GRCm38.p4 is proposed; exact donor substrain, transcript/patch equivalence and the study’s auxiliary ERCC version remain unverified. Such interpretation assets are not required for generic lossless FASTQ compression.</t>
+          <t>Acquire both listed archive ends and verify integrity and pairing. Keep the exact chosen FASTQ representation and order. Same-species GRCm39 is proposed; exact donor substrain, transcript/patch equivalence and the study’s auxiliary ERCC version remain unverified. Such interpretation assets are not required for generic lossless FASTQ compression.</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
@@ -33429,7 +33880,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>The proposed reference is Renan, not Thatcher; exact read/reference matching remains unverified. Nominal paired 150-base sequencing is documented, but actual FASTQ lengths, qualities, headers and integrity have not been examined.</t>
+          <t>The proposed reference is Chinese Spring, not Thatcher; exact read/reference matching remains unverified. Nominal paired 150-base sequencing is documented, but actual FASTQ lengths, qualities, headers and integrity have not been examined.</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -39349,7 +39800,7 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>Official assembly metadata identifiesTriticum_aestivum_Renan_v2.1,GCA_937894285.1,assemblydate2022-0</t>
+          <t>Official assembly metadata identifiesTriticum_aestivum_Renan_v2.1,GCF_018294505.1,assemblydate2022-0</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
@@ -39364,7 +39815,7 @@
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>Official assembly metadata identifiesTriticum_aestivum_Renan_v2.1,GCA_937894285.1,assemblydate2022-08.</t>
+          <t>Official assembly metadata identifiesTriticum_aestivum_Renan_v2.1,GCF_018294505.1,assemblydate2022-08.</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
@@ -40633,12 +41084,12 @@
       </c>
       <c r="E104" s="3" t="inlineStr">
         <is>
-          <t>This ordinary wheat resequencing run adds a large, polyploid crop genome. Both FASTQ ends of one Thatcher sample are included. The primary study reports about 542.5 billion bases and 35× coverage for this sample; this is a real study input, not a subset made to reach a benchmark size. The proposed Renan assembly is from the same species but a different cultivar.</t>
+          <t>This ordinary wheat resequencing run adds a large, polyploid crop genome. Both FASTQ ends of one Thatcher sample are included. The primary study reports about 542.5 billion bases and 35× coverage for this sample; this is a real study input, not a subset made to reach a benchmark size. The proposed Chinese Spring assembly is from the same species but a different cultivar.</t>
         </is>
       </c>
       <c r="F104" s="3" t="inlineStr">
         <is>
-          <t>The proposed reference is Renan, not Thatcher; exact read/reference matching remains unverified. Nominal paired 150-base sequencing is documented, but actual FASTQ lengths, qualities, headers and integrity have not been examined.</t>
+          <t>The proposed reference is Chinese Spring, not Thatcher; exact read/reference matching remains unverified. Nominal paired 150-base sequencing is documented, but actual FASTQ lengths, qualities, headers and integrity have not been examined.</t>
         </is>
       </c>
       <c r="G104" s="3" t="inlineStr">

</xml_diff>